<commit_message>
ci(dev): publish dev build from d65fabed451d21be93d5b1a8760a46d9ffc2f5e7 d65fabed451d21be93d5b1a8760a46d9ffc2f5e7
</commit_message>
<xml_diff>
--- a/dev/CodeSystem-PSCED.xlsx
+++ b/dev/CodeSystem-PSCED.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.0</t>
+    <t>0.2.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-01T03:34:09+00:00</t>
+    <t>2026-04-01T03:44:59+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>